<commit_message>
Inventario: tipo de evento "Plaga" y emergencia agropecuaria por tucura de 2009
- formulario.json y XLSForm suman PLAGUE (guía de DesInventar); el formulario
  de Kobo se desplegó con la opción nueva.
- Registro 0038, aprobado por Sebastián: Ordenanza 6769/2009 (homologa el
  Decreto 2185/09).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014b9JyNPWpHa7PqfWpjXmux
</commit_message>
<xml_diff>
--- a/datos/inventario/formulario_inventario.xlsx
+++ b/datos/inventario/formulario_inventario.xlsx
@@ -72,7 +72,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Registrá un evento adverso ocurrido en el partido de Necochea o una vulnerabilidad observada, tal como lo informó un medio. Cada registro se revisa antes de publicarse en el mapa de riesgos (https://jsbertole-ai.github.io/mapa-riesgos-necochea/). No cargues nombres de personas ni domicilios particulares. Este formulario no pide tus datos; KoboToolbox guarda en su historial interno la dirección IP de cada envío, que el proyecto no exporta ni publica.</t>
+          <t xml:space="preserve">**Registrá un evento adverso ocurrido en el partido de Necochea o una vulnerabilidad observada, tal como lo informó un medio local o nacional, un organismo oficial, o una causa o un fallo judicial.** Cada registro se revisa antes de publicarse en el mapa para la gestión del riesgo. No cargues nombres de personas ni domicilios particulares. Este formulario no pide tus datos; KoboToolbox guarda en su historial interno la dirección IP de cada envío, que el proyecto no exporta ni publica.</t>
         </is>
       </c>
     </row>
@@ -929,12 +929,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medio que publicó la nota</t>
+          <t xml:space="preserve">Fuente: medio, organismo o tribunal</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Escribilo siempre de la misma forma, para poder agrupar los registros por medio.</t>
+          <t xml:space="preserve">Escribila siempre de la misma forma, para poder agrupar los registros. En un fallo, el tribunal y la sala.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -956,12 +956,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Título de la nota</t>
+          <t xml:space="preserve">Título de la nota o del documento, o número de causa</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sirve para revisar el registro; no se publica.</t>
+          <t xml:space="preserve">De una causa, solo el número: no copies la carátula, porque suele traer nombres de personas. Sirve para revisar el registro; no se publica.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fecha de publicación de la nota</t>
+          <t xml:space="preserve">Fecha de publicación o del fallo</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enlace a la nota</t>
+          <t xml:space="preserve">Enlace a la fuente</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1479,29 +1479,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">OTHER</t>
+          <t xml:space="preserve">PLAGUE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Otro</t>
+          <t xml:space="preserve">Plaga (proliferación de insectos u otros animales que dañan cultivos, ganado o personas)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">tipo_vulnerabilidad</t>
+          <t xml:space="preserve">tipo_evento</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">desague</t>
+          <t xml:space="preserve">OTHER</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Desagüe pluvial obstruido o insuficiente</t>
+          <t xml:space="preserve">Otro</t>
         </is>
       </c>
     </row>
@@ -1513,12 +1513,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">zona_anegable</t>
+          <t xml:space="preserve">desague</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Viviendas o servicios en zona que se anega</t>
+          <t xml:space="preserve">Desagüe pluvial obstruido o insuficiente</t>
         </is>
       </c>
     </row>
@@ -1530,12 +1530,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">erosion</t>
+          <t xml:space="preserve">zona_anegable</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Erosión costera, de barrancas o de márgenes</t>
+          <t xml:space="preserve">Viviendas o servicios en zona que se anega</t>
         </is>
       </c>
     </row>
@@ -1547,12 +1547,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">basural</t>
+          <t xml:space="preserve">erosion</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Basural o quema a cielo abierto</t>
+          <t xml:space="preserve">Erosión costera, de barrancas o de márgenes</t>
         </is>
       </c>
     </row>
@@ -1564,12 +1564,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">infraestructura</t>
+          <t xml:space="preserve">basural</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Infraestructura deteriorada (puente, camino, edificio público)</t>
+          <t xml:space="preserve">Basural o quema a cielo abierto</t>
         </is>
       </c>
     </row>
@@ -1581,12 +1581,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">peligrosas</t>
+          <t xml:space="preserve">infraestructura</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Almacenamiento o transporte de sustancias peligrosas</t>
+          <t xml:space="preserve">Infraestructura deteriorada (puente, camino, edificio público)</t>
         </is>
       </c>
     </row>
@@ -1598,12 +1598,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">combustible</t>
+          <t xml:space="preserve">peligrosas</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pastizal seco o falta de cortafuegos</t>
+          <t xml:space="preserve">Almacenamiento o transporte de sustancias peligrosas</t>
         </is>
       </c>
     </row>
@@ -1615,12 +1615,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">arbolado</t>
+          <t xml:space="preserve">combustible</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Árboles o postes con riesgo de caída</t>
+          <t xml:space="preserve">Pastizal seco o falta de cortafuegos</t>
         </is>
       </c>
     </row>
@@ -1632,29 +1632,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">otra</t>
+          <t xml:space="preserve">arbolado</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Otra</t>
+          <t xml:space="preserve">Árboles o postes con riesgo de caída</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">localidad</t>
+          <t xml:space="preserve">tipo_vulnerabilidad</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">necochea_quequen</t>
+          <t xml:space="preserve">otra</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Necochea y Quequén</t>
+          <t xml:space="preserve">Otra</t>
         </is>
       </c>
     </row>
@@ -1666,12 +1666,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">juan_n_fernandez</t>
+          <t xml:space="preserve">necochea_quequen</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Juan N. Fernández</t>
+          <t xml:space="preserve">Necochea y Quequén</t>
         </is>
       </c>
     </row>
@@ -1683,12 +1683,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">nicanor_olivera</t>
+          <t xml:space="preserve">juan_n_fernandez</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nicanor Olivera (La Dulce)</t>
+          <t xml:space="preserve">Juan N. Fernández</t>
         </is>
       </c>
     </row>
@@ -1700,12 +1700,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">energia</t>
+          <t xml:space="preserve">nicanor_olivera</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Energía</t>
+          <t xml:space="preserve">Nicanor Olivera (La Dulce)</t>
         </is>
       </c>
     </row>
@@ -1717,12 +1717,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">claraz</t>
+          <t xml:space="preserve">energia</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Claraz</t>
+          <t xml:space="preserve">Energía</t>
         </is>
       </c>
     </row>
@@ -1734,12 +1734,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">ramon_santamarina</t>
+          <t xml:space="preserve">claraz</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ramón Santamarina</t>
+          <t xml:space="preserve">Claraz</t>
         </is>
       </c>
     </row>
@@ -1751,29 +1751,29 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">rural</t>
+          <t xml:space="preserve">ramon_santamarina</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zona rural o costa fuera de las localidades</t>
+          <t xml:space="preserve">Ramón Santamarina</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">servicio</t>
+          <t xml:space="preserve">localidad</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">transporte</t>
+          <t xml:space="preserve">rural</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transporte (calles, rutas, ferrocarril, puentes, muelles)</t>
+          <t xml:space="preserve">Zona rural o costa fuera de las localidades</t>
         </is>
       </c>
     </row>
@@ -1785,12 +1785,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">comunicaciones</t>
+          <t xml:space="preserve">transporte</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comunicaciones (telefonía, radio, televisión, internet)</t>
+          <t xml:space="preserve">Transporte (calles, rutas, ferrocarril, puentes, muelles)</t>
         </is>
       </c>
     </row>
@@ -1802,12 +1802,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">energia</t>
+          <t xml:space="preserve">comunicaciones</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Energía (electricidad, gas, combustibles)</t>
+          <t xml:space="preserve">Comunicaciones (telefonía, radio, televisión, internet)</t>
         </is>
       </c>
     </row>
@@ -1819,12 +1819,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">acueducto</t>
+          <t xml:space="preserve">energia</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Agua potable</t>
+          <t xml:space="preserve">Energía (electricidad, gas, combustibles)</t>
         </is>
       </c>
     </row>
@@ -1836,12 +1836,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">alcantarillado</t>
+          <t xml:space="preserve">acueducto</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cloacas y desagües pluviales</t>
+          <t xml:space="preserve">Agua potable</t>
         </is>
       </c>
     </row>
@@ -1853,12 +1853,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">educacion</t>
+          <t xml:space="preserve">alcantarillado</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Educación</t>
+          <t xml:space="preserve">Cloacas y desagües pluviales</t>
         </is>
       </c>
     </row>
@@ -1870,12 +1870,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">salud</t>
+          <t xml:space="preserve">educacion</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Salud</t>
+          <t xml:space="preserve">Educación</t>
         </is>
       </c>
     </row>
@@ -1887,12 +1887,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">socorro</t>
+          <t xml:space="preserve">salud</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instalaciones de socorro (bomberos, Defensa Civil)</t>
+          <t xml:space="preserve">Salud</t>
         </is>
       </c>
     </row>
@@ -1904,12 +1904,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">agropecuario</t>
+          <t xml:space="preserve">socorro</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Agropecuario</t>
+          <t xml:space="preserve">Instalaciones de socorro (bomberos, Defensa Civil)</t>
         </is>
       </c>
     </row>
@@ -1921,12 +1921,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">industrias</t>
+          <t xml:space="preserve">agropecuario</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Industrias</t>
+          <t xml:space="preserve">Agropecuario</t>
         </is>
       </c>
     </row>
@@ -1938,10 +1938,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t xml:space="preserve">industrias</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrias</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">servicio</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t xml:space="preserve">otros</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t xml:space="preserve">Otros</t>
         </is>

</xml_diff>

<commit_message>
Formulario de Kobo simplificado (31 a 15 preguntas) y fecha en día/mes/año; el inventario acepta registros sin medio ni fecha de la fuente; caché v98
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014b9JyNPWpHa7PqfWpjXmux
</commit_message>
<xml_diff>
--- a/datos/inventario/formulario_inventario.xlsx
+++ b/datos/inventario/formulario_inventario.xlsx
@@ -72,7 +72,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">**Registrá un evento adverso ocurrido en el partido de Necochea o una vulnerabilidad observada, tal como lo informó un medio local o nacional, un organismo oficial, o una causa o un fallo judicial.** Cada registro se revisa antes de publicarse en el mapa para la gestión del riesgo. No cargues nombres de personas ni domicilios particulares. Este formulario no pide tus datos; KoboToolbox guarda en su historial interno la dirección IP de cada envío, que el proyecto no exporta ni publica.</t>
+          <t xml:space="preserve">**Registrá un evento adverso ocurrido en el partido de Necochea o una vulnerabilidad observada, tal como lo informó un medio local o nacional, un organismo oficial, o una causa o un fallo judicial.** Cada registro se revisa antes de publicarse en el mapa para la gestión del riesgo. No cargues nombres de personas. Este formulario no pide tus datos; KoboToolbox guarda en su historial interno la dirección IP de cada envío, que el proyecto no exporta ni publica.</t>
         </is>
       </c>
     </row>
@@ -101,7 +101,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">date</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -114,6 +114,11 @@
           <t xml:space="preserve">Fecha del evento o de la observación</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Día/mes/año, por ejemplo 13/04/2015.</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
@@ -121,12 +126,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">. &lt;= today() and . &gt;= date('1900-01-01')</t>
+          <t xml:space="preserve">regex(., '^(0?[1-9]|[12][0-9]|3[01])/(0?[1-9]|1[0-2])/(19|20)[0-9]{2}$')</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t xml:space="preserve">La fecha tiene que estar entre 1900 y hoy.</t>
+          <t xml:space="preserve">Escribila como día/mes/año, por ejemplo 13/04/2015.</t>
         </is>
       </c>
     </row>
@@ -224,12 +229,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Barrio, paraje o lugar público (opcional)</t>
+          <t xml:space="preserve">Lugar (opcional)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Por ejemplo: barrio, esquina, puente, escuela. Nunca un domicilio particular.</t>
+          <t xml:space="preserve">Barrio, dirección, esquina o lugar público, como lo nombra la nota.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -261,34 +266,49 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marcalo solo si la nota nombra un lugar público concreto. Si no, dejalo vacío: alcanza con la localidad.</t>
+          <t xml:space="preserve">Marcá el lugar que nombra la nota. Si no nombra ninguno, dejalo vacío: alcanza con la localidad.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">note</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">nota_efectos</t>
+          <t xml:space="preserve">descripcion</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Efectos, según la nota (opcional)</t>
+          <t xml:space="preserve">¿Qué pasó?</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cargá solo las cifras que da la nota. Un campo vacío significa sin dato, no cero.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
+          <t xml:space="preserve">En pocas líneas y con tus palabras.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">string-length(.) &lt;= 400</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Máximo 400 caracteres.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">multiline</t>
         </is>
       </c>
     </row>
@@ -305,12 +325,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Muertos</t>
+          <t xml:space="preserve">Muertos (opcional)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personas fallecidas por causas directas. Si la cifra no está confirmada oficialmente, anotala en las observaciones de efectos.</t>
+          <t xml:space="preserve">Solo si la nota da la cifra.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -337,17 +357,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">desaparecidos</t>
+          <t xml:space="preserve">heridos</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Desaparecidos</t>
+          <t xml:space="preserve">Heridos o enfermos (opcional)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personas cuyo paradero es desconocido. No se suman a los muertos.</t>
+          <t xml:space="preserve">Solo si la nota da la cifra.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -374,17 +394,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">heridos</t>
+          <t xml:space="preserve">evacuados</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Heridos o enfermos</t>
+          <t xml:space="preserve">Evacuados (opcional)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personas afectadas en su salud o integridad física por causa directa del evento.</t>
+          <t xml:space="preserve">Solo si la nota da la cifra.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -406,22 +426,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">integer</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">damnificados</t>
+          <t xml:space="preserve">observaciones_efectos</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Damnificados</t>
+          <t xml:space="preserve">Otras cifras que da la nota (opcional)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personas con grave daño en sus bienes o servicios (por ejemplo, vivienda destruida). Incluye reubicados.</t>
+          <t xml:space="preserve">Por ejemplo: viviendas afectadas, hectáreas, cortes de servicios.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -431,626 +451,69 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve">. &gt;= 0</t>
+          <t xml:space="preserve">string-length(.) &lt;= 300</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
+          <t xml:space="preserve">Máximo 300 caracteres.</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">multiline</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">integer</t>
+          <t xml:space="preserve">text</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">afectados</t>
+          <t xml:space="preserve">fuente_url</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Afectados</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Personas, distintas de los damnificados, con efectos indirectos: cortes de servicios, aislamiento, pérdida de trabajo.</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
+          <t xml:space="preserve">Enlace a la nota o a la fuente</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve">. &gt;= 0</t>
+          <t xml:space="preserve">regex(., '^https?://.+')</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
+          <t xml:space="preserve">Tiene que ser un enlace que empiece con http:// o https://</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">integer</t>
+          <t xml:space="preserve">acknowledge</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">evacuados</t>
+          <t xml:space="preserve">licencia</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evacuados</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Personas evacuadas temporalmente de viviendas, trabajos, escuelas u hospitales.</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">reubicados</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reubicados</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Personas trasladadas de forma permanente a otro lugar de vivienda.</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">viviendas_destruidas</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Viviendas destruidas</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Viviendas que quedaron inhabitables.</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">viviendas_afectadas</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Viviendas afectadas</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Viviendas con daños menores, que siguen siendo habitables. No se suman a las destruidas.</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">centros_educativos</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Centros educativos afectados</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Escuelas, jardines, institutos. Incluye los usados como albergue.</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">centros_salud</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Centros de salud afectados</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Salas, clínicas y hospitales dañados o afectados.</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">vias_m</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vías afectadas (metros)</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Longitud de calles, caminos o rutas destruidas o inhabilitadas, solo si la nota la da en metros o kilómetros.</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">decimal</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cultivos_ha</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cultivos, pastizales o bosques (hectáreas)</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Superficie afectada, solo si la nota la da en hectáreas.</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un número mayor o igual a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">integer</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ganado</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ganado perdido (cabezas)</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Animales perdidos: bovinos, porcinos, ovinos, aves.</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &gt;= 0</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un número entero mayor o igual a cero.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">observaciones_efectos</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Observaciones de efectos (opcional)</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cifras en familias (no las pases a personas), cifras no confirmadas o diferencias entre fuentes.</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">string-length(.) &lt;= 300</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Máximo 300 caracteres.</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">multiline</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">select_multiple servicio</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicios_afectados</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Servicios o sectores afectados (opcional)</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">${tipo_registro} = 'evento'</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">descripcion</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Descripción breve</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Qué pasó y dónde, en pocas líneas y con tus palabras. Sin nombres de personas ni domicilios.</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">string-length(.) &lt;= 400</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Máximo 400 caracteres.</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">multiline</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fuente_medio</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fuente: medio, organismo o tribunal</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Escribila siempre de la misma forma, para poder agrupar los registros. En un fallo, el tribunal y la sala.</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fuente_titulo</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Título de la nota o del documento, o número de causa</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">De una causa, solo el número: no copies la carátula, porque suele traer nombres de personas. Sirve para revisar el registro; no se publica.</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">date</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fuente_fecha</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fecha de publicación o del fallo</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">. &lt;= today()</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">La fecha no puede ser posterior a hoy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">text</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">fuente_url</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Enlace a la fuente</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">regex(., '^https?://.+')</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tiene que ser un enlace que empiece con http:// o https://</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">acknowledge</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">licencia</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
           <t xml:space="preserve">Acepto que este registro se publique con licencia Creative Commons Atribución 4.0 (CC BY 4.0), citado como "Inventario local de eventos y vulnerabilidades del partido de Necochea".</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t xml:space="preserve">yes</t>
         </is>
@@ -1777,193 +1240,6 @@
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">transporte</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Transporte (calles, rutas, ferrocarril, puentes, muelles)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">comunicaciones</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Comunicaciones (telefonía, radio, televisión, internet)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">energia</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Energía (electricidad, gas, combustibles)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">acueducto</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agua potable</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">alcantarillado</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cloacas y desagües pluviales</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">educacion</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Educación</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">salud</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Salud</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">socorro</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Instalaciones de socorro (bomberos, Defensa Civil)</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">agropecuario</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Agropecuario</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">industrias</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Industrias</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">servicio</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">otros</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Otros</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>